<commit_message>
feat(F-NAR-016): TREE-DIF-065 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-065.xlsx
+++ b/stories/arbres/TREE-DIF-065.xlsx
@@ -16511,7 +16511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16554,6 +16554,20 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>